<commit_message>
efat: coba uji skenario
</commit_message>
<xml_diff>
--- a/code_notebooks/implementasi/waktu_komputasi_skenario.xlsx
+++ b/code_notebooks/implementasi/waktu_komputasi_skenario.xlsx
@@ -452,10 +452,10 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>6125.4</v>
+        <v>470.78</v>
       </c>
       <c r="C2" t="n">
-        <v>14.95</v>
+        <v>8.59</v>
       </c>
     </row>
     <row r="3">
@@ -465,10 +465,10 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>517</v>
+        <v>666.41</v>
       </c>
       <c r="C3" t="n">
-        <v>2.16</v>
+        <v>2.42</v>
       </c>
     </row>
     <row r="4">
@@ -478,10 +478,10 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>10894.63</v>
+        <v>19654.88</v>
       </c>
       <c r="C4" t="n">
-        <v>25.62</v>
+        <v>11.96</v>
       </c>
     </row>
     <row r="5">
@@ -491,10 +491,10 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>109540.86</v>
+        <v>150757.86</v>
       </c>
       <c r="C5" t="n">
-        <v>3.06</v>
+        <v>2.1</v>
       </c>
     </row>
     <row r="6">
@@ -504,10 +504,10 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>27591.53</v>
+        <v>28900.13</v>
       </c>
       <c r="C6" t="n">
-        <v>54.15</v>
+        <v>25.38</v>
       </c>
     </row>
     <row r="7">
@@ -517,10 +517,10 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>27775.2</v>
+        <v>29238.19</v>
       </c>
       <c r="C7" t="n">
-        <v>45.87</v>
+        <v>24.23</v>
       </c>
     </row>
     <row r="8">
@@ -530,10 +530,10 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>31680.97</v>
+        <v>34164.08</v>
       </c>
       <c r="C8" t="n">
-        <v>47.36</v>
+        <v>25.48</v>
       </c>
     </row>
     <row r="9">
@@ -543,10 +543,10 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>93526.42</v>
+        <v>119505.66</v>
       </c>
       <c r="C9" t="n">
-        <v>46.87</v>
+        <v>25.21</v>
       </c>
     </row>
   </sheetData>

</xml_diff>